<commit_message>
Agrega campos crudos de activos/componentes a subcomponentes y carpeta DIPLAN_INPUTS
- Subcomponentes: la matriz y la evidencia ahora incluyen el texto crudo del que
  se extraen las palabras clave (activos_f7 de Rep_Activos_F7 y
  componentes_inversion de HR Inversiones) para que se pueda replicar y mejorar
  la identificacion. Diccionario con fuente de palabras clave y regla.
- Insumos reorganizados en carpeta DIPLAN_INPUTS para facil identificacion;
  los 3 scripts apuntan a DIPLAN_INPUTS (insumos) y DIPLAN_OUTPUT (resultados).
- README actualizado con la estructura y la lista de inputs.
</commit_message>
<xml_diff>
--- a/DIPLAN_OUTPUT/base_final/subcomponentes_total_diccionario.xlsx
+++ b/DIPLAN_OUTPUT/base_final/subcomponentes_total_diccionario.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -434,7 +434,17 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>activos_clave</t>
+          <t>palabras_clave</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>fuente_palabras_clave</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>regla</t>
         </is>
       </c>
     </row>
@@ -459,6 +469,16 @@
           <t>demolicion, edificacion, obras exteriores</t>
         </is>
       </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Rep_Activos_F7 (campo ACTIVO) + HR Inversiones (DES_PRODUCTO/DES_ACCION/DES_TIPO_COMPONENTE)</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>cumple=1 si alguna palabra clave aparece en activos_f7 o componentes_inversion del cod_local</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -481,6 +501,16 @@
           <t>demolicion, edificacion</t>
         </is>
       </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Rep_Activos_F7 (campo ACTIVO) + HR Inversiones (DES_PRODUCTO/DES_ACCION/DES_TIPO_COMPONENTE)</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>cumple=1 si alguna palabra clave aparece en activos_f7 o componentes_inversion del cod_local</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -503,6 +533,16 @@
           <t>reforzamiento, muro de contencion, estructura</t>
         </is>
       </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Rep_Activos_F7 (campo ACTIVO) + HR Inversiones (DES_PRODUCTO/DES_ACCION/DES_TIPO_COMPONENTE)</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>cumple=1 si alguna palabra clave aparece en activos_f7 o componentes_inversion del cod_local</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -525,6 +565,16 @@
           <t>modulo, prefabricad, provisional, contingen</t>
         </is>
       </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Rep_Activos_F7 (campo ACTIVO) + HR Inversiones (DES_PRODUCTO/DES_ACCION/DES_TIPO_COMPONENTE)</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>cumple=1 si alguna palabra clave aparece en activos_f7 o componentes_inversion del cod_local</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -547,6 +597,16 @@
           <t>cerco perimetrico, cerco</t>
         </is>
       </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Rep_Activos_F7 (campo ACTIVO) + HR Inversiones (DES_PRODUCTO/DES_ACCION/DES_TIPO_COMPONENTE)</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>cumple=1 si alguna palabra clave aparece en activos_f7 o componentes_inversion del cod_local</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -569,6 +629,16 @@
           <t>agua, desague, saneamiento, ubs, unidades basicas, reservorio, captacion, linea de conduccion, red de distribucion, pozo, tanque, letrina, biodigestor</t>
         </is>
       </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Rep_Activos_F7 (campo ACTIVO) + HR Inversiones (DES_PRODUCTO/DES_ACCION/DES_TIPO_COMPONENTE)</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>cumple=1 si alguna palabra clave aparece en activos_f7 o componentes_inversion del cod_local</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -591,6 +661,16 @@
           <t>servicios higienicos, vestidor, cisterna, tanque elevado, planta de tratamiento, agua potable, ptar</t>
         </is>
       </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Rep_Activos_F7 (campo ACTIVO) + HR Inversiones (DES_PRODUCTO/DES_ACCION/DES_TIPO_COMPONENTE)</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>cumple=1 si alguna palabra clave aparece en activos_f7 o componentes_inversion del cod_local</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -613,6 +693,16 @@
           <t>electric, energia, subestacion, panel solar, red electrica, tablero, instalacion electrica</t>
         </is>
       </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Rep_Activos_F7 (campo ACTIVO) + HR Inversiones (DES_PRODUCTO/DES_ACCION/DES_TIPO_COMPONENTE)</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>cumple=1 si alguna palabra clave aparece en activos_f7 o componentes_inversion del cod_local</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -635,6 +725,16 @@
           <t>mobiliario, equipamiento, equipo, mueble, carpeta, pizarra, computo</t>
         </is>
       </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Rep_Activos_F7 (campo ACTIVO) + HR Inversiones (DES_PRODUCTO/DES_ACCION/DES_TIPO_COMPONENTE)</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>cumple=1 si alguna palabra clave aparece en activos_f7 o componentes_inversion del cod_local</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -657,6 +757,16 @@
           <t>piso, pavimento, vereda, cobertura, pintura, carpinteria, acabado, cuneta, sardinel, techo</t>
         </is>
       </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Rep_Activos_F7 (campo ACTIVO) + HR Inversiones (DES_PRODUCTO/DES_ACCION/DES_TIPO_COMPONENTE)</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>cumple=1 si alguna palabra clave aparece en activos_f7 o componentes_inversion del cod_local</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -679,6 +789,16 @@
           <t>edificacion, aula, ambiente, pabellon, taller, laboratorio</t>
         </is>
       </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Rep_Activos_F7 (campo ACTIVO) + HR Inversiones (DES_PRODUCTO/DES_ACCION/DES_TIPO_COMPONENTE)</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>cumple=1 si alguna palabra clave aparece en activos_f7 o componentes_inversion del cod_local</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -701,6 +821,16 @@
           <t>reforzamiento, estructura, muro de contencion</t>
         </is>
       </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Rep_Activos_F7 (campo ACTIVO) + HR Inversiones (DES_PRODUCTO/DES_ACCION/DES_TIPO_COMPONENTE)</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>cumple=1 si alguna palabra clave aparece en activos_f7 o componentes_inversion del cod_local</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -723,6 +853,16 @@
           <t>edificacion, aula, modulo</t>
         </is>
       </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Rep_Activos_F7 (campo ACTIVO) + HR Inversiones (DES_PRODUCTO/DES_ACCION/DES_TIPO_COMPONENTE)</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>cumple=1 si alguna palabra clave aparece en activos_f7 o componentes_inversion del cod_local</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -745,6 +885,16 @@
           <t>electric, energia, panel solar, subestacion, red electrica</t>
         </is>
       </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Rep_Activos_F7 (campo ACTIVO) + HR Inversiones (DES_PRODUCTO/DES_ACCION/DES_TIPO_COMPONENTE)</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>cumple=1 si alguna palabra clave aparece en activos_f7 o componentes_inversion del cod_local</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -767,6 +917,16 @@
           <t>rampa, accesibilidad, ascensor, elevador, baranda, pasamano</t>
         </is>
       </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Rep_Activos_F7 (campo ACTIVO) + HR Inversiones (DES_PRODUCTO/DES_ACCION/DES_TIPO_COMPONENTE)</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>cumple=1 si alguna palabra clave aparece en activos_f7 o componentes_inversion del cod_local</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -789,6 +949,16 @@
           <t>edificacion, aula, ambiente, pabellon, infraestructura, usos multiples, taller, laboratorio</t>
         </is>
       </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Rep_Activos_F7 (campo ACTIVO) + HR Inversiones (DES_PRODUCTO/DES_ACCION/DES_TIPO_COMPONENTE)</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>cumple=1 si alguna palabra clave aparece en activos_f7 o componentes_inversion del cod_local</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -809,6 +979,16 @@
       <c r="D18" t="inlineStr">
         <is>
           <t>saneamiento fisico legal, fisico legal, intangible, otras acciones de intangibles, titulacion</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Rep_Activos_F7 (campo ACTIVO) + HR Inversiones (DES_PRODUCTO/DES_ACCION/DES_TIPO_COMPONENTE)</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>cumple=1 si alguna palabra clave aparece en activos_f7 o componentes_inversion del cod_local</t>
         </is>
       </c>
     </row>

</xml_diff>